<commit_message>
moved configuration out of lib
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/testgetattributeasjson.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/testgetattributeasjson.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rce7001dd3f7247ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra27194c6271f4272"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
     <x:row r="2">
       <x:c r="B2" t="s">
@@ -127,7 +127,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fcc2d930b1b487a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b79b2d1827c48fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
added test for configuration strategies
</commit_message>
<xml_diff>
--- a/Tests/Test Config From EXCEL/testdata/testgetattributeasjson.xlsx
+++ b/Tests/Test Config From EXCEL/testdata/testgetattributeasjson.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra27194c6271f4272"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5f44b586a8734fff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,7 +127,7 @@
     </x:row>
   </x:sheetData>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b79b2d1827c48fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R485f0def04e54df9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>